<commit_message>
Fix bypass resistor, add missing Vcc. Move to Kicad-9
</commit_message>
<xml_diff>
--- a/Combined-BOM.xlsx
+++ b/Combined-BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git-repos\Equalizer-8-band\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5A88FE0-B07D-4DDF-AC0F-7DDA07449C4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6BF8C2B-86E3-4713-9D38-32708B571B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1350" yWindow="870" windowWidth="31365" windowHeight="21675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5460" yWindow="5460" windowWidth="31290" windowHeight="14400" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main-Board-BOM" sheetId="2" r:id="rId1"/>
@@ -23,10 +23,21 @@
     <definedName name="ExternalData_1" localSheetId="1" hidden="1">'4-Row-POT-BOM'!$A$1:$F$4</definedName>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">'Main-Board-BOM'!$A$1:$F$34</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -539,7 +550,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -552,6 +566,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -571,13 +598,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="20">
@@ -2110,7 +2141,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074AAD50-1887-4242-B494-38133E085B4F}">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -3318,11 +3349,33 @@
         <v>10</v>
       </c>
     </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B56" s="1">
+        <v>11.74</v>
+      </c>
+    </row>
+    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B57" s="1">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B58" s="1">
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="59" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B59" s="2">
+        <f>SUM(B56:B58)</f>
+        <v>14.87</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>